<commit_message>
Add Imam mobile account to UAT package
</commit_message>
<xml_diff>
--- a/artifacts/uat/UAT_LOGISTIK_END_TO_END_TESTER.xlsx
+++ b/artifacts/uat/UAT_LOGISTIK_END_TO_END_TESTER.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Akun Tester" sheetId="1" r:id="R6c10dea0bb5f4c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Checklist UAT" sheetId="2" r:id="Rb502b9a047a145f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Ringkasan" sheetId="3" r:id="R57636c812bb241cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Akun Tester" sheetId="1" r:id="R213c0d2399d945f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Checklist UAT" sheetId="2" r:id="R997cccf13ae4449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Ringkasan" sheetId="3" r:id="R0d630e9cfab5463a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -487,10 +487,33 @@
         <x:v>Jika akun tidak ada setelah reset, buat dari Supir -&gt; Akses Mobile.</x:v>
       </x:c>
     </x:row>
+    <x:row r="10" ht="64.5" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>Portal Driver / Mobile Driver</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>DRIVER - Imam</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>imam@driver</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>driver12345</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>/driver/login dan app mobile</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str">
+        <x:v>UAT case Imam: trip baru setelah DO lama selesai, input SJ/barang dari mobile.</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="str">
+        <x:v>Password sudah di-reset untuk UAT pada 2026-05-13.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra03d467bee46417a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R154e98fb6dfd49c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5321,7 +5344,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61b80bd85fc3435f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a0701773c0847f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5443,7 +5466,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f1557ac2f884123"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R872912361fb745b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>